<commit_message>
fix(data): store Abhaar Vastram's number the way the column stores numbers
Their mobile sat in the master sheet as the text "99799-40730" while every
other number in the column is a plain numeric cell, so it sorted and matched
differently from its neighbours. Write it as 9979940730.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013qWPnMZpCQ1UxTmqa4iLhA
</commit_message>
<xml_diff>
--- a/STE_data_sheet.xlsx
+++ b/STE_data_sheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rebel\OneDrive\Documents\Projects\STE-feature-clean-code-assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BD09DE3-9E0D-43AB-AB27-E990B4EE6A06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BB15C91-0DCC-401B-A990-A19E5E10657E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="12196" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="8" windowWidth="19395" windowHeight="12194" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ste-final-list" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="361" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="248">
   <si>
     <t>Brand Name</t>
   </si>
@@ -69,9 +69,6 @@
   </si>
   <si>
     <t>Sarees</t>
-  </si>
-  <si>
-    <t>99799-40730</t>
   </si>
   <si>
     <t xml:space="preserve">Abhilasha Enterprises </t>
@@ -1674,16 +1671,16 @@
         <f t="shared" si="0"/>
         <v>3m x 12m</v>
       </c>
-      <c r="E4" s="13" t="s">
-        <v>11</v>
+      <c r="E4" s="13">
+        <v>9979940730</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="12" t="s">
         <v>12</v>
-      </c>
-      <c r="B5" s="12" t="s">
-        <v>13</v>
       </c>
       <c r="C5" s="13">
         <v>100</v>
@@ -1698,7 +1695,7 @@
     </row>
     <row r="6" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B6" s="9" t="s">
         <v>10</v>
@@ -1716,10 +1713,10 @@
     </row>
     <row r="7" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="9" t="s">
         <v>15</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>16</v>
       </c>
       <c r="C7" s="10">
         <v>1000</v>
@@ -1729,12 +1726,12 @@
         <v>3m x 30m</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="11" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B8" s="12" t="s">
         <v>10</v>
@@ -1752,10 +1749,10 @@
     </row>
     <row r="9" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" s="9" t="s">
         <v>19</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>20</v>
       </c>
       <c r="C9" s="10">
         <v>400</v>
@@ -1765,12 +1762,12 @@
         <v>3m x 12m</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="11" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B10" s="12" t="s">
         <v>6</v>
@@ -1788,10 +1785,10 @@
     </row>
     <row r="11" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" s="9" t="s">
         <v>23</v>
-      </c>
-      <c r="B11" s="9" t="s">
-        <v>24</v>
       </c>
       <c r="C11" s="10">
         <v>100</v>
@@ -1806,7 +1803,7 @@
     </row>
     <row r="12" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="11" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B12" s="12" t="s">
         <v>10</v>
@@ -1819,12 +1816,12 @@
         <v>3m x 3m</v>
       </c>
       <c r="E12" s="13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B13" s="9" t="s">
         <v>6</v>
@@ -1842,7 +1839,7 @@
     </row>
     <row r="14" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="8" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B14" s="9" t="s">
         <v>10</v>
@@ -1860,7 +1857,7 @@
     </row>
     <row r="15" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="11" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B15" s="12" t="s">
         <v>10</v>
@@ -1878,10 +1875,10 @@
     </row>
     <row r="16" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="B16" s="12" t="s">
         <v>30</v>
-      </c>
-      <c r="B16" s="12" t="s">
-        <v>31</v>
       </c>
       <c r="C16" s="13">
         <v>100</v>
@@ -1896,7 +1893,7 @@
     </row>
     <row r="17" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B17" s="9" t="s">
         <v>10</v>
@@ -1914,10 +1911,10 @@
     </row>
     <row r="18" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="B18" s="12" t="s">
         <v>33</v>
-      </c>
-      <c r="B18" s="12" t="s">
-        <v>34</v>
       </c>
       <c r="C18" s="13">
         <v>1000</v>
@@ -1932,10 +1929,10 @@
     </row>
     <row r="19" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C19" s="10">
         <v>100</v>
@@ -1950,7 +1947,7 @@
     </row>
     <row r="20" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B20" s="9" t="s">
         <v>10</v>
@@ -1963,15 +1960,15 @@
         <v>3m x 12m</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="B21" s="15" t="s">
         <v>38</v>
-      </c>
-      <c r="B21" s="15" t="s">
-        <v>39</v>
       </c>
       <c r="C21" s="16">
         <v>200</v>
@@ -1986,7 +1983,7 @@
     </row>
     <row r="22" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B22" s="9" t="s">
         <v>6</v>
@@ -2004,10 +2001,10 @@
     </row>
     <row r="23" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="B23" s="12" t="s">
         <v>41</v>
-      </c>
-      <c r="B23" s="12" t="s">
-        <v>42</v>
       </c>
       <c r="C23" s="13">
         <v>100</v>
@@ -2022,7 +2019,7 @@
     </row>
     <row r="24" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B24" s="9" t="s">
         <v>10</v>
@@ -2040,10 +2037,10 @@
     </row>
     <row r="25" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B25" s="12" t="s">
         <v>44</v>
-      </c>
-      <c r="B25" s="12" t="s">
-        <v>45</v>
       </c>
       <c r="C25" s="13">
         <v>400</v>
@@ -2053,12 +2050,12 @@
         <v>3m x 12m</v>
       </c>
       <c r="E25" s="13" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B26" s="9" t="s">
         <v>10</v>
@@ -2076,7 +2073,7 @@
     </row>
     <row r="27" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="11" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B27" s="12" t="s">
         <v>10</v>
@@ -2094,16 +2091,16 @@
     </row>
     <row r="28" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="40" t="s">
+        <v>245</v>
+      </c>
+      <c r="B28" s="41" t="s">
         <v>246</v>
-      </c>
-      <c r="B28" s="41" t="s">
-        <v>247</v>
       </c>
       <c r="C28" s="42">
         <v>100</v>
       </c>
       <c r="D28" s="42" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E28" s="42">
         <v>8200203732</v>
@@ -2111,10 +2108,10 @@
     </row>
     <row r="29" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="8" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C29" s="10">
         <v>200</v>
@@ -2129,7 +2126,7 @@
     </row>
     <row r="30" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="11" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B30" s="9" t="s">
         <v>10</v>
@@ -2147,7 +2144,7 @@
     </row>
     <row r="31" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="11" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B31" s="12" t="s">
         <v>10</v>
@@ -2160,15 +2157,15 @@
         <v>3m x 18m</v>
       </c>
       <c r="E31" s="13" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C32" s="10">
         <v>200</v>
@@ -2178,15 +2175,15 @@
         <v>3m x 6m</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B33" s="9" t="s">
         <v>55</v>
-      </c>
-      <c r="B33" s="9" t="s">
-        <v>56</v>
       </c>
       <c r="C33" s="10">
         <v>800</v>
@@ -2201,7 +2198,7 @@
     </row>
     <row r="34" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="32" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B34" s="33" t="s">
         <v>10</v>
@@ -2219,7 +2216,7 @@
     </row>
     <row r="35" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="35" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B35" s="35" t="s">
         <v>10</v>
@@ -2228,7 +2225,7 @@
         <v>200</v>
       </c>
       <c r="D35" s="36" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E35" s="36">
         <v>8980835552</v>
@@ -2236,7 +2233,7 @@
     </row>
     <row r="36" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="29" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B36" s="30" t="s">
         <v>10</v>
@@ -2254,10 +2251,10 @@
     </row>
     <row r="37" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="11" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B37" s="12" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C37" s="13">
         <v>400</v>
@@ -2272,10 +2269,10 @@
     </row>
     <row r="38" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B38" s="9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C38" s="10">
         <v>1000</v>
@@ -2285,15 +2282,15 @@
         <v>3m x 30m</v>
       </c>
       <c r="E38" s="10" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="B39" s="12" t="s">
         <v>62</v>
-      </c>
-      <c r="B39" s="12" t="s">
-        <v>63</v>
       </c>
       <c r="C39" s="13">
         <v>200</v>
@@ -2308,7 +2305,7 @@
     </row>
     <row r="40" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="11" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B40" s="12" t="s">
         <v>10</v>
@@ -2317,7 +2314,7 @@
         <v>200</v>
       </c>
       <c r="D40" s="13" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E40" s="13">
         <v>9601700354</v>
@@ -2325,10 +2322,10 @@
     </row>
     <row r="41" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="11" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B41" s="12" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C41" s="13">
         <v>600</v>
@@ -2343,7 +2340,7 @@
     </row>
     <row r="42" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="8" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B42" s="9" t="s">
         <v>6</v>
@@ -2361,7 +2358,7 @@
     </row>
     <row r="43" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B43" s="12" t="s">
         <v>10</v>
@@ -2379,7 +2376,7 @@
     </row>
     <row r="44" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B44" s="9" t="s">
         <v>10</v>
@@ -2397,10 +2394,10 @@
     </row>
     <row r="45" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="B45" s="9" t="s">
         <v>68</v>
-      </c>
-      <c r="B45" s="9" t="s">
-        <v>69</v>
       </c>
       <c r="C45" s="10">
         <v>300</v>
@@ -2410,15 +2407,15 @@
         <v>3m x 9m</v>
       </c>
       <c r="E45" s="10" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="46" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="B46" s="9" t="s">
         <v>71</v>
-      </c>
-      <c r="B46" s="9" t="s">
-        <v>72</v>
       </c>
       <c r="C46" s="17">
         <v>300</v>
@@ -2428,15 +2425,15 @@
         <v>3m x 9m</v>
       </c>
       <c r="E46" s="17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="47" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="B47" s="12" t="s">
         <v>74</v>
-      </c>
-      <c r="B47" s="12" t="s">
-        <v>75</v>
       </c>
       <c r="C47" s="18">
         <v>300</v>
@@ -2451,7 +2448,7 @@
     </row>
     <row r="48" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48" s="8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B48" s="9" t="s">
         <v>10</v>
@@ -2469,10 +2466,10 @@
     </row>
     <row r="49" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="B49" s="9" t="s">
         <v>77</v>
-      </c>
-      <c r="B49" s="9" t="s">
-        <v>78</v>
       </c>
       <c r="C49" s="10">
         <v>200</v>
@@ -2487,7 +2484,7 @@
     </row>
     <row r="50" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A50" s="29" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B50" s="37" t="s">
         <v>6</v>
@@ -2496,7 +2493,7 @@
         <v>200</v>
       </c>
       <c r="D50" s="38" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E50" s="39">
         <v>98988666093</v>
@@ -2504,10 +2501,10 @@
     </row>
     <row r="51" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A51" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="B51" s="12" t="s">
         <v>79</v>
-      </c>
-      <c r="B51" s="12" t="s">
-        <v>80</v>
       </c>
       <c r="C51" s="13">
         <v>1200</v>
@@ -2517,12 +2514,12 @@
         <v>3m x 36m</v>
       </c>
       <c r="E51" s="13" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="52" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A52" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B52" s="9" t="s">
         <v>10</v>
@@ -2535,12 +2532,12 @@
         <v>3m x 9m</v>
       </c>
       <c r="E52" s="10" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="53" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A53" s="8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B53" s="9" t="s">
         <v>6</v>
@@ -2558,10 +2555,10 @@
     </row>
     <row r="54" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A54" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="B54" s="12" t="s">
         <v>85</v>
-      </c>
-      <c r="B54" s="12" t="s">
-        <v>86</v>
       </c>
       <c r="C54" s="13">
         <v>400</v>
@@ -2576,10 +2573,10 @@
     </row>
     <row r="55" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A55" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="B55" s="12" t="s">
         <v>87</v>
-      </c>
-      <c r="B55" s="12" t="s">
-        <v>88</v>
       </c>
       <c r="C55" s="13">
         <v>200</v>
@@ -2594,7 +2591,7 @@
     </row>
     <row r="56" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A56" s="11" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B56" s="12" t="s">
         <v>10</v>
@@ -2612,7 +2609,7 @@
     </row>
     <row r="57" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A57" s="8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B57" s="9" t="s">
         <v>10</v>
@@ -2630,7 +2627,7 @@
     </row>
     <row r="58" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A58" s="14" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B58" s="15" t="s">
         <v>10</v>
@@ -2643,12 +2640,12 @@
         <v>3m x 18m</v>
       </c>
       <c r="E58" s="16" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="59" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A59" s="8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B59" s="9" t="s">
         <v>6</v>
@@ -2661,15 +2658,15 @@
         <v>3m x 9m</v>
       </c>
       <c r="E59" s="10" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="60" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A60" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="B60" s="12" t="s">
         <v>95</v>
-      </c>
-      <c r="B60" s="12" t="s">
-        <v>96</v>
       </c>
       <c r="C60" s="13">
         <v>200</v>
@@ -2684,7 +2681,7 @@
     </row>
     <row r="61" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A61" s="8" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B61" s="9" t="s">
         <v>10</v>
@@ -2702,7 +2699,7 @@
     </row>
     <row r="62" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A62" s="8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B62" s="9" t="s">
         <v>10</v>
@@ -2720,7 +2717,7 @@
     </row>
     <row r="63" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A63" s="20" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B63" s="21" t="s">
         <v>6</v>
@@ -2733,15 +2730,15 @@
         <v>3m x 18m</v>
       </c>
       <c r="E63" s="22" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="64" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A64" s="11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B64" s="12" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C64" s="13">
         <v>300</v>
@@ -2751,15 +2748,15 @@
         <v>3m x 9m</v>
       </c>
       <c r="E64" s="13" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="65" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A65" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="B65" s="9" t="s">
         <v>103</v>
-      </c>
-      <c r="B65" s="9" t="s">
-        <v>104</v>
       </c>
       <c r="C65" s="10">
         <v>100</v>
@@ -2769,12 +2766,12 @@
         <v>3m x 3m</v>
       </c>
       <c r="E65" s="10" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="66" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A66" s="11" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B66" s="12" t="s">
         <v>6</v>
@@ -2792,10 +2789,10 @@
     </row>
     <row r="67" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A67" s="8" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B67" s="9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C67" s="10">
         <v>400</v>
@@ -2805,12 +2802,12 @@
         <v>3m x 12m</v>
       </c>
       <c r="E67" s="10" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="68" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A68" s="11" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B68" s="12" t="s">
         <v>10</v>
@@ -2823,15 +2820,15 @@
         <v>3m x 18m</v>
       </c>
       <c r="E68" s="13" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="69" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A69" s="11" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B69" s="12" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C69" s="13">
         <v>100</v>
@@ -2846,7 +2843,7 @@
     </row>
     <row r="70" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A70" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B70" s="9" t="s">
         <v>10</v>
@@ -2864,7 +2861,7 @@
     </row>
     <row r="71" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A71" s="8" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B71" s="9" t="s">
         <v>6</v>
@@ -2877,12 +2874,12 @@
         <v>3m x 6m</v>
       </c>
       <c r="E71" s="10" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="72" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A72" s="8" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B72" s="9" t="s">
         <v>10</v>
@@ -2900,7 +2897,7 @@
     </row>
     <row r="73" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A73" s="11" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B73" s="12" t="s">
         <v>10</v>
@@ -2913,15 +2910,15 @@
         <v>3m x 9m</v>
       </c>
       <c r="E73" s="13" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="74" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A74" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="B74" s="9" t="s">
         <v>118</v>
-      </c>
-      <c r="B74" s="9" t="s">
-        <v>119</v>
       </c>
       <c r="C74" s="10">
         <v>600</v>
@@ -2931,15 +2928,15 @@
         <v>3m x 18m</v>
       </c>
       <c r="E74" s="10" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="75" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A75" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="B75" s="12" t="s">
         <v>121</v>
-      </c>
-      <c r="B75" s="12" t="s">
-        <v>122</v>
       </c>
       <c r="C75" s="13">
         <v>1000</v>
@@ -2954,10 +2951,10 @@
     </row>
     <row r="76" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A76" s="11" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B76" s="12" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C76" s="13">
         <v>100</v>
@@ -2972,24 +2969,24 @@
     </row>
     <row r="77" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A77" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="B77" s="9" t="s">
         <v>124</v>
-      </c>
-      <c r="B77" s="9" t="s">
-        <v>125</v>
       </c>
       <c r="C77" s="10">
         <v>2000</v>
       </c>
       <c r="D77" s="10" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E77" s="10" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="78" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A78" s="11" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B78" s="12" t="s">
         <v>10</v>
@@ -3007,10 +3004,10 @@
     </row>
     <row r="79" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A79" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B79" s="12" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C79" s="13">
         <v>100</v>
@@ -3020,12 +3017,12 @@
         <v>3m x 3m</v>
       </c>
       <c r="E79" s="13" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="80" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A80" s="11" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B80" s="12" t="s">
         <v>10</v>
@@ -3043,7 +3040,7 @@
     </row>
     <row r="81" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A81" s="8" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B81" s="9" t="s">
         <v>10</v>
@@ -3061,7 +3058,7 @@
     </row>
     <row r="82" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A82" s="11" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B82" s="12" t="s">
         <v>10</v>
@@ -3079,10 +3076,10 @@
     </row>
     <row r="83" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A83" s="11" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B83" s="12" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C83" s="13">
         <v>200</v>
@@ -3097,7 +3094,7 @@
     </row>
     <row r="84" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A84" s="8" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B84" s="9" t="s">
         <v>6</v>
@@ -3115,10 +3112,10 @@
     </row>
     <row r="85" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A85" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="B85" s="9" t="s">
         <v>135</v>
-      </c>
-      <c r="B85" s="9" t="s">
-        <v>136</v>
       </c>
       <c r="C85" s="10">
         <v>200</v>
@@ -3133,7 +3130,7 @@
     </row>
     <row r="86" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A86" s="8" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B86" s="9" t="s">
         <v>6</v>
@@ -3151,10 +3148,10 @@
     </row>
     <row r="87" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A87" s="8" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B87" s="9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C87" s="10">
         <v>100</v>
@@ -3169,10 +3166,10 @@
     </row>
     <row r="88" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A88" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="B88" s="9" t="s">
         <v>139</v>
-      </c>
-      <c r="B88" s="9" t="s">
-        <v>140</v>
       </c>
       <c r="C88" s="10">
         <v>200</v>
@@ -3182,12 +3179,12 @@
         <v>3m x 6m</v>
       </c>
       <c r="E88" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="89" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A89" s="11" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B89" s="12" t="s">
         <v>10</v>
@@ -3200,15 +3197,15 @@
         <v>3m x 9m</v>
       </c>
       <c r="E89" s="13" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="90" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A90" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="B90" s="9" t="s">
         <v>144</v>
-      </c>
-      <c r="B90" s="9" t="s">
-        <v>145</v>
       </c>
       <c r="C90" s="10">
         <v>400</v>
@@ -3218,12 +3215,12 @@
         <v>3m x 12m</v>
       </c>
       <c r="E90" s="10" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="91" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A91" s="11" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B91" s="12" t="s">
         <v>6</v>
@@ -3236,15 +3233,15 @@
         <v>3m x 12m</v>
       </c>
       <c r="E91" s="23" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="92" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A92" s="8" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B92" s="9" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C92" s="10">
         <v>300</v>
@@ -3259,10 +3256,10 @@
     </row>
     <row r="93" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A93" s="11" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B93" s="12" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C93" s="13">
         <v>400</v>
@@ -3272,12 +3269,12 @@
         <v>3m x 12m</v>
       </c>
       <c r="E93" s="13" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="94" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A94" s="8" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B94" s="9" t="s">
         <v>6</v>
@@ -3295,10 +3292,10 @@
     </row>
     <row r="95" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A95" s="11" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B95" s="12" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C95" s="13">
         <v>600</v>
@@ -3313,16 +3310,16 @@
     </row>
     <row r="96" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A96" s="40" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B96" s="41" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C96" s="42">
         <v>600</v>
       </c>
       <c r="D96" s="42" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="E96" s="42">
         <v>9374072626</v>
@@ -3330,7 +3327,7 @@
     </row>
     <row r="97" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A97" s="8" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B97" s="9" t="s">
         <v>10</v>
@@ -3348,7 +3345,7 @@
     </row>
     <row r="98" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A98" s="11" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B98" s="12" t="s">
         <v>10</v>
@@ -3366,10 +3363,10 @@
     </row>
     <row r="99" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A99" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="B99" s="9" t="s">
         <v>156</v>
-      </c>
-      <c r="B99" s="9" t="s">
-        <v>157</v>
       </c>
       <c r="C99" s="10">
         <v>600</v>
@@ -3384,7 +3381,7 @@
     </row>
     <row r="100" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A100" s="11" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B100" s="12" t="s">
         <v>6</v>
@@ -3402,7 +3399,7 @@
     </row>
     <row r="101" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A101" s="8" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B101" s="9" t="s">
         <v>10</v>
@@ -3420,7 +3417,7 @@
     </row>
     <row r="102" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A102" s="11" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B102" s="12" t="s">
         <v>6</v>
@@ -3438,10 +3435,10 @@
     </row>
     <row r="103" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A103" s="11" t="s">
+        <v>160</v>
+      </c>
+      <c r="B103" s="12" t="s">
         <v>161</v>
-      </c>
-      <c r="B103" s="12" t="s">
-        <v>162</v>
       </c>
       <c r="C103" s="13">
         <v>600</v>
@@ -3456,10 +3453,10 @@
     </row>
     <row r="104" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A104" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="B104" s="9" t="s">
         <v>163</v>
-      </c>
-      <c r="B104" s="9" t="s">
-        <v>164</v>
       </c>
       <c r="C104" s="10">
         <v>100</v>
@@ -3474,10 +3471,10 @@
     </row>
     <row r="105" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A105" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="B105" s="12" t="s">
         <v>165</v>
-      </c>
-      <c r="B105" s="12" t="s">
-        <v>166</v>
       </c>
       <c r="C105" s="13">
         <v>100</v>
@@ -3492,10 +3489,10 @@
     </row>
     <row r="106" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A106" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B106" s="9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C106" s="10">
         <v>200</v>
@@ -3510,7 +3507,7 @@
     </row>
     <row r="107" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A107" s="11" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B107" s="12" t="s">
         <v>6</v>
@@ -3528,7 +3525,7 @@
     </row>
     <row r="108" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A108" s="8" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B108" s="9" t="s">
         <v>10</v>
@@ -3546,7 +3543,7 @@
     </row>
     <row r="109" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A109" s="11" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B109" s="12" t="s">
         <v>10</v>
@@ -3564,7 +3561,7 @@
     </row>
     <row r="110" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A110" s="11" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B110" s="12" t="s">
         <v>10</v>
@@ -3573,13 +3570,13 @@
         <v>2600</v>
       </c>
       <c r="D110" s="13" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E110" s="43"/>
     </row>
     <row r="111" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A111" s="8" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B111" s="9" t="s">
         <v>10</v>
@@ -3592,15 +3589,15 @@
         <v>3m x 18m</v>
       </c>
       <c r="E111" s="10" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="112" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A112" s="11" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B112" s="12" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C112" s="13">
         <v>300</v>
@@ -3610,12 +3607,12 @@
         <v>3m x 9m</v>
       </c>
       <c r="E112" s="23" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="113" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A113" s="8" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B113" s="9" t="s">
         <v>10</v>
@@ -3633,10 +3630,10 @@
     </row>
     <row r="114" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A114" s="11" t="s">
+        <v>176</v>
+      </c>
+      <c r="B114" s="12" t="s">
         <v>177</v>
-      </c>
-      <c r="B114" s="12" t="s">
-        <v>178</v>
       </c>
       <c r="C114" s="13">
         <v>400</v>
@@ -3651,7 +3648,7 @@
     </row>
     <row r="115" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A115" s="11" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B115" s="12" t="s">
         <v>10</v>
@@ -3664,12 +3661,12 @@
         <v>3m x 6m</v>
       </c>
       <c r="E115" s="13" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="116" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A116" s="8" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B116" s="9" t="s">
         <v>10</v>
@@ -3687,7 +3684,7 @@
     </row>
     <row r="117" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A117" s="8" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B117" s="9" t="s">
         <v>10</v>
@@ -3700,15 +3697,15 @@
         <v>3m x 3m</v>
       </c>
       <c r="E117" s="10" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="118" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A118" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="B118" s="9" t="s">
         <v>184</v>
-      </c>
-      <c r="B118" s="9" t="s">
-        <v>185</v>
       </c>
       <c r="C118" s="10">
         <v>200</v>
@@ -3723,10 +3720,10 @@
     </row>
     <row r="119" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A119" s="11" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B119" s="12" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C119" s="13">
         <v>200</v>
@@ -3741,10 +3738,10 @@
     </row>
     <row r="120" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A120" s="11" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B120" s="12" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C120" s="13">
         <v>100</v>
@@ -3759,7 +3756,7 @@
     </row>
     <row r="121" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A121" s="11" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B121" s="12" t="s">
         <v>10</v>
@@ -3772,12 +3769,12 @@
         <v>3m x 30m</v>
       </c>
       <c r="E121" s="13" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="122" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A122" s="8" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B122" s="9" t="s">
         <v>6</v>
@@ -3790,15 +3787,15 @@
         <v>3m x 3m</v>
       </c>
       <c r="E122" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="123" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A123" s="11" t="s">
+        <v>191</v>
+      </c>
+      <c r="B123" s="12" t="s">
         <v>192</v>
-      </c>
-      <c r="B123" s="12" t="s">
-        <v>193</v>
       </c>
       <c r="C123" s="13">
         <v>600</v>
@@ -3808,12 +3805,12 @@
         <v>3m x 18m</v>
       </c>
       <c r="E123" s="13" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="124" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A124" s="8" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B124" s="9" t="s">
         <v>6</v>
@@ -3831,7 +3828,7 @@
     </row>
     <row r="125" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A125" s="11" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B125" s="12" t="s">
         <v>6</v>
@@ -3849,7 +3846,7 @@
     </row>
     <row r="126" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A126" s="11" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B126" s="12" t="s">
         <v>6</v>
@@ -3862,15 +3859,15 @@
         <v>3m x 6m</v>
       </c>
       <c r="E126" s="13" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="127" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A127" s="8" t="s">
+        <v>198</v>
+      </c>
+      <c r="B127" s="9" t="s">
         <v>199</v>
-      </c>
-      <c r="B127" s="9" t="s">
-        <v>200</v>
       </c>
       <c r="C127" s="10">
         <v>600</v>
@@ -3880,12 +3877,12 @@
         <v>3m x 18m</v>
       </c>
       <c r="E127" s="10" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="128" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A128" s="11" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B128" s="12" t="s">
         <v>10</v>
@@ -3903,7 +3900,7 @@
     </row>
     <row r="129" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A129" s="14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B129" s="15" t="s">
         <v>10</v>
@@ -3916,12 +3913,12 @@
         <v>3m x 12m</v>
       </c>
       <c r="E129" s="16" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="130" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A130" s="8" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B130" s="9" t="s">
         <v>10</v>
@@ -3939,7 +3936,7 @@
     </row>
     <row r="131" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A131" s="8" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B131" s="9" t="s">
         <v>10</v>
@@ -3952,12 +3949,12 @@
         <v>3m x 12m</v>
       </c>
       <c r="E131" s="10" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="132" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A132" s="8" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B132" s="9" t="s">
         <v>6</v>
@@ -3975,10 +3972,10 @@
     </row>
     <row r="133" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A133" s="11" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B133" s="12" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C133" s="13">
         <v>1000</v>
@@ -3988,12 +3985,12 @@
         <v>3m x 30m</v>
       </c>
       <c r="E133" s="13" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="134" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A134" s="11" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B134" s="12" t="s">
         <v>6</v>
@@ -4011,7 +4008,7 @@
     </row>
     <row r="135" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A135" s="11" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B135" s="12" t="s">
         <v>6</v>
@@ -4024,12 +4021,12 @@
         <v>3m x 12m</v>
       </c>
       <c r="E135" s="13" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="136" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A136" s="8" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B136" s="9" t="s">
         <v>10</v>
@@ -4042,12 +4039,12 @@
         <v>3m x 9m</v>
       </c>
       <c r="E136" s="10" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="137" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A137" s="11" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B137" s="12" t="s">
         <v>10</v>
@@ -4065,7 +4062,7 @@
     </row>
     <row r="138" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A138" s="11" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B138" s="12" t="s">
         <v>6</v>
@@ -4083,10 +4080,10 @@
     </row>
     <row r="139" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A139" s="8" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B139" s="9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C139" s="10">
         <v>400</v>
@@ -4096,15 +4093,15 @@
         <v>3m x 12m</v>
       </c>
       <c r="E139" s="10" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="140" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A140" s="11" t="s">
+        <v>218</v>
+      </c>
+      <c r="B140" s="12" t="s">
         <v>219</v>
-      </c>
-      <c r="B140" s="12" t="s">
-        <v>220</v>
       </c>
       <c r="C140" s="13">
         <v>200</v>
@@ -4114,12 +4111,12 @@
         <v>3m x 6m</v>
       </c>
       <c r="E140" s="13" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="141" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A141" s="8" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B141" s="9" t="s">
         <v>10</v>
@@ -4137,10 +4134,10 @@
     </row>
     <row r="142" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A142" s="11" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B142" s="12" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C142" s="13">
         <v>200</v>
@@ -4155,7 +4152,7 @@
     </row>
     <row r="143" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A143" s="11" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B143" s="12" t="s">
         <v>6</v>
@@ -4173,10 +4170,10 @@
     </row>
     <row r="144" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A144" s="8" t="s">
+        <v>224</v>
+      </c>
+      <c r="B144" s="9" t="s">
         <v>225</v>
-      </c>
-      <c r="B144" s="9" t="s">
-        <v>226</v>
       </c>
       <c r="C144" s="10">
         <v>200</v>
@@ -4186,12 +4183,12 @@
         <v>3m x 6m</v>
       </c>
       <c r="E144" s="10" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="145" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A145" s="11" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B145" s="12" t="s">
         <v>10</v>
@@ -4209,10 +4206,10 @@
     </row>
     <row r="146" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A146" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B146" s="9" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C146" s="10">
         <v>100</v>
@@ -4222,12 +4219,12 @@
         <v>3m x 3m</v>
       </c>
       <c r="E146" s="10" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="147" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A147" s="8" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B147" s="9" t="s">
         <v>6</v>
@@ -4240,12 +4237,12 @@
         <v>3m x 9m</v>
       </c>
       <c r="E147" s="10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="148" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A148" s="8" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B148" s="9" t="s">
         <v>6</v>
@@ -4263,7 +4260,7 @@
     </row>
     <row r="149" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A149" s="24" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B149" s="25" t="s">
         <v>10</v>
@@ -4281,10 +4278,10 @@
     </row>
     <row r="150" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A150" s="5" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B150" s="5" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C150" s="18">
         <v>800</v>
@@ -4299,10 +4296,10 @@
     </row>
     <row r="151" spans="1:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A151" s="5" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B151" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C151" s="18">
         <v>400</v>

</xml_diff>